<commit_message>
Amplía la capa a actividad comercial (comercios + servicios)
- descargar_comercio.py: además de shop=* y mercados, incluye servicios comerciales
  (gastronomía, bancos/finanzas, farmacias, combustible, cines), oficinas (office=*)
  y talleres/oficios (craft=*) de OSM. Nuevas categorías en el tooltip.
- Cobertura: 6.287 → 10.342 puntos; expuestos en zona de inundación 34 → 73
  (gastronomía 13, oficinas 12, minorista 18, alimentos 9, talleres 8, etc.).
- Excel comercio_riesgo.xlsx, mapa (leyenda/pie), y KPI del panel actualizados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/exposicion/comercio_riesgo.xlsx
+++ b/datos/exposicion/comercio_riesgo.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Comercio en riesgo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comercio en riesgo'!$A$4:$E$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comercio en riesgo'!$A$4:$E$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -733,76 +733,76 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>(sin nombre)</t>
+          <t>Integral: Villa Hayes</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Comercio (sin especificar)</t>
+          <t>Combustible</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>fuel</t>
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>-25.25586</v>
+        <v>-25.10285</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>-57.639</v>
+        <v>-57.54294</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Las Palomas</t>
+          <t>Integral: Villa Hayes</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Comercio (sin especificar)</t>
+          <t>Combustible</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>fuel</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>-25.18372</v>
+        <v>-25.10329</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-57.53869</v>
+        <v>-57.54233</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Molino San Luis</t>
+          <t>Shell Ita Enrramada</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Comercio (sin especificar)</t>
+          <t>Combustible</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>fuel</t>
         </is>
       </c>
       <c r="D16" s="7" t="n">
-        <v>-25.27574</v>
+        <v>-25.35912</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>-57.60991</v>
+        <v>-57.6445</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>SAMU/CELL</t>
+          <t>(sin nombre)</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -816,85 +816,85 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>-25.26547</v>
+        <v>-25.25586</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-57.60613</v>
+        <v>-57.639</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>(sin nombre)</t>
+          <t>Las Palomas</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Comercio minorista</t>
+          <t>Comercio (sin especificar)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>electronics</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D18" s="7" t="n">
-        <v>-25.27449</v>
+        <v>-25.18372</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>-57.60772</v>
+        <v>-57.53869</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>(sin nombre)</t>
+          <t>Molino San Luis</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Comercio minorista</t>
+          <t>Comercio (sin especificar)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>storage_rental</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>-25.27091</v>
+        <v>-25.27574</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-57.60735</v>
+        <v>-57.60991</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>(sin nombre)</t>
+          <t>SAMU/CELL</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Comercio minorista</t>
+          <t>Comercio (sin especificar)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D20" s="7" t="n">
-        <v>-25.27066</v>
+        <v>-25.26547</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>-57.60533</v>
+        <v>-57.60613</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Baga S.A.</t>
+          <t>(sin nombre)</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -904,20 +904,20 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>storage_rental</t>
+          <t>electronics</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>-25.27275</v>
+        <v>-25.27449</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-57.60885</v>
+        <v>-57.60772</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Centro Visual</t>
+          <t>(sin nombre)</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -927,20 +927,20 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>optician</t>
+          <t>storage_rental</t>
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>-25.27433</v>
+        <v>-25.27091</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>-57.60744</v>
+        <v>-57.60735</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Costas del Río</t>
+          <t>(sin nombre)</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -950,20 +950,20 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>fishing</t>
+          <t>car</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>-25.25572</v>
+        <v>-25.27066</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-57.63895</v>
+        <v>-57.60533</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Nike Factory Store</t>
+          <t>Baga S.A.</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -973,20 +973,20 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>shoes</t>
+          <t>storage_rental</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>-25.27507</v>
+        <v>-25.27275</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>-57.61014</v>
+        <v>-57.60885</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Centro Visual</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -996,20 +996,20 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>mobile_phone</t>
+          <t>optician</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>-25.30971</v>
+        <v>-25.27433</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-57.66706</v>
+        <v>-57.60744</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Pescaderia</t>
+          <t>Costas del Río</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1023,16 +1023,16 @@
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>-25.18413</v>
+        <v>-25.25572</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>-57.53552</v>
+        <v>-57.63895</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Pescaderia Andresito</t>
+          <t>Nike Factory Store</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1042,20 +1042,20 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>fishing</t>
+          <t>shoes</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>-25.18446</v>
+        <v>-25.27507</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-57.53894</v>
+        <v>-57.61014</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Printstore - Multigraph</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>printer_ink</t>
+          <t>mobile_phone</t>
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>-25.27386</v>
+        <v>-25.30971</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>-57.60724</v>
+        <v>-57.66706</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Regalería Nenita</t>
+          <t>Pescaderia</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1088,20 +1088,20 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>gift</t>
+          <t>fishing</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>-25.2504</v>
+        <v>-25.18413</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>-57.64002</v>
+        <v>-57.53552</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Salón de belleza</t>
+          <t>Pescaderia Andresito</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -1111,20 +1111,20 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>beauty</t>
+          <t>fishing</t>
         </is>
       </c>
       <c r="D30" s="7" t="n">
-        <v>-25.2559</v>
+        <v>-25.18446</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>-57.63897</v>
+        <v>-57.53894</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Taller de automoviles</t>
+          <t>Printstore - Multigraph</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1134,20 +1134,20 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>car_repair</t>
+          <t>printer_ink</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>-25.25337</v>
+        <v>-25.27386</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-57.63764</v>
+        <v>-57.60724</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Taller de lanchas</t>
+          <t>Regalería Nenita</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1157,20 +1157,20 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>car_repair</t>
+          <t>gift</t>
         </is>
       </c>
       <c r="D32" s="7" t="n">
-        <v>-25.25289</v>
+        <v>-25.2504</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>-57.63949</v>
+        <v>-57.64002</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Tienda de ropas</t>
+          <t>Salón de belleza</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1180,20 +1180,20 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>clothes</t>
+          <t>beauty</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>-25.25187</v>
+        <v>-25.2559</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>-57.64103</v>
+        <v>-57.63897</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Zavidoro Corporations NIKE</t>
+          <t>Taller de automoviles</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -1203,20 +1203,20 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>sports</t>
+          <t>car_repair</t>
         </is>
       </c>
       <c r="D34" s="7" t="n">
-        <v>-25.35743</v>
+        <v>-25.25337</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>-57.64304</v>
+        <v>-57.63764</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Zion Francis Wake School</t>
+          <t>Taller de lanchas</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1226,87 +1226,984 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>outdoor</t>
+          <t>car_repair</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>-25.35697</v>
+        <v>-25.25289</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>-57.64447</v>
+        <v>-57.63949</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Autoservice Thiago</t>
+          <t>Tienda de ropas</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Gran superficie</t>
+          <t>Comercio minorista</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>supermarket</t>
+          <t>clothes</t>
         </is>
       </c>
       <c r="D36" s="7" t="n">
-        <v>-25.28006</v>
+        <v>-25.25187</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>-57.62333</v>
+        <v>-57.64103</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Biggie</t>
+          <t>Zavidoro Corporations NIKE</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Gran superficie</t>
+          <t>Comercio minorista</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>supermarket</t>
+          <t>sports</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>-25.27421</v>
+        <v>-25.35743</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>-57.60782</v>
+        <v>-57.64304</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t>Zion Francis Wake School</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Comercio minorista</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>outdoor</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>-25.35697</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>-57.64447</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Farmacia Vicente Scavone</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>pharmacy</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>-25.27485</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>-57.60853</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>-25.18282</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>-57.5395</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>-25.18283</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>-57.53968</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>-25.18296</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>-57.53925</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>-25.18284</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>-57.53982</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>-25.18273</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>-57.53924</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Comedor Ña Cata</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>-25.2547</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>-57.63822</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>El Cacique</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>-25.35893</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>-57.64518</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Havanna Cafe</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>cafe</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>-25.27312</v>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>-57.60794</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Heladería</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>ice_cream</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>-25.25604</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>-57.63924</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Heladería y Mercería JyJ</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>ice_cream</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>-25.2342</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>-57.63129</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Integral Go: Villa Hayes</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>-25.10291</v>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>-57.54194</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Pollería</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>fast_food</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>-25.25581</v>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>-57.63908</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Shopping del Pescado</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Gastronomía</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>-25.18286</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>-57.54107</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Autoservice Thiago</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Gran superficie</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>supermarket</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="n">
+        <v>-25.28006</v>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>-57.62333</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Biggie</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Gran superficie</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>supermarket</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>-25.27421</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>-57.60782</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
           <t>Petersen</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Gran superficie</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>mall</t>
         </is>
       </c>
-      <c r="D38" s="7" t="n">
+      <c r="D55" s="5" t="n">
         <v>-25.27379</v>
       </c>
-      <c r="E38" s="7" t="n">
+      <c r="E55" s="5" t="n">
         <v>-57.60631</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>architect</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>-25.27339</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>-57.60862</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Aduana Ita Enramada</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>customs</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="n">
+        <v>-25.36102</v>
+      </c>
+      <c r="E57" s="5" t="n">
+        <v>-57.64578</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Centro Avanzado de Control de Tráfico</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>-25.27765</v>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>-57.63135</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Datalab</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="n">
+        <v>-25.27343</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>-57.6076</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Estudio Jurídico</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>notary</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>-25.25482</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>-57.64118</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Industria Nacional del Cemento</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="n">
+        <v>-25.49762</v>
+      </c>
+      <c r="E61" s="5" t="n">
+        <v>-57.5632</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Justicia Electoral</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>-25.25313</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>-57.64113</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Juzgado de Paz de Chaco'i</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>courthouse</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="n">
+        <v>-25.25396</v>
+      </c>
+      <c r="E63" s="5" t="n">
+        <v>-57.64119</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Oficina de Diseño Gráfico</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>advertising_agency</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>-25.25178</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>-57.64116</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Partido Liberal</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>political_party</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="n">
+        <v>-25.2532</v>
+      </c>
+      <c r="E65" s="5" t="n">
+        <v>-57.64097</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Policia Nacional Departamento de Seguridad Urbana y Turística</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>administrative</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>-25.27753</v>
+      </c>
+      <c r="E66" s="7" t="n">
+        <v>-57.62228</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Puerto Caacupemi</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Oficina / servicios</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>customs</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="n">
+        <v>-25.22592</v>
+      </c>
+      <c r="E67" s="5" t="n">
+        <v>-57.57137</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Lavadero de automóviles</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Servicios comerciales</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>car_wash</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>-25.25193</v>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>-57.64001</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Itaú</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Servicios financieros</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>-25.27161</v>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>-57.6051</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>pottery</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>-25.2379</v>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>-57.63283</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>pottery</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="n">
+        <v>-25.23806</v>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>-57.63253</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>pottery</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>-25.23801</v>
+      </c>
+      <c r="E72" s="7" t="n">
+        <v>-57.63302</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>(sin nombre)</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>pottery</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="n">
+        <v>-25.2375</v>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>-57.63263</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Antigua Fábrica de Cerámica</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>pottery</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>-25.23774</v>
+      </c>
+      <c r="E74" s="7" t="n">
+        <v>-57.63249</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>Herrería Alberto Franco</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>blacksmith</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="n">
+        <v>-25.25166</v>
+      </c>
+      <c r="E75" s="5" t="n">
+        <v>-57.64142</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Modista</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>dressmaker</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>-25.25232</v>
+      </c>
+      <c r="E76" s="7" t="n">
+        <v>-57.6414</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>Pintor</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Taller / oficio</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>painter</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="n">
+        <v>-25.2509</v>
+      </c>
+      <c r="E77" s="5" t="n">
+        <v>-57.63896</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E38"/>
+  <autoFilter ref="A4:E77"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>

</xml_diff>